<commit_message>
refactor: improve error handling and validation in product import forms
</commit_message>
<xml_diff>
--- a/storage/app/public/import/pharmacy_product_import_template.xlsx
+++ b/storage/app/public/import/pharmacy_product_import_template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="31">
   <si>
     <t>product_code</t>
   </si>
@@ -91,16 +91,19 @@
     <t>Acme Pharma</t>
   </si>
   <si>
+    <t>pc</t>
+  </si>
+  <si>
+    <t>2027-12-31</t>
+  </si>
+  <si>
+    <t>BATCH-001</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
     <t>tablet</t>
-  </si>
-  <si>
-    <t>2027-12-31</t>
-  </si>
-  <si>
-    <t>BATCH-001</t>
-  </si>
-  <si>
-    <t>no</t>
   </si>
   <si>
     <t>Pain relief medication</t>
@@ -488,24 +491,24 @@
   <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="11" max="11" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="20.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="17" max="17" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="18" max="18" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="17.567" customWidth="true" style="0"/>
+    <col min="2" max="2" width="15.139" customWidth="true" style="0"/>
+    <col min="3" max="3" width="17.567" customWidth="true" style="0"/>
+    <col min="4" max="4" width="10.426" customWidth="true" style="0"/>
+    <col min="5" max="5" width="17.567" customWidth="true" style="0"/>
+    <col min="6" max="6" width="13.997" customWidth="true" style="0"/>
+    <col min="7" max="7" width="8.141" customWidth="true" style="0"/>
+    <col min="8" max="8" width="15.139" customWidth="true" style="0"/>
+    <col min="9" max="9" width="15.139" customWidth="true" style="0"/>
+    <col min="10" max="10" width="18.71" customWidth="true" style="0"/>
+    <col min="11" max="11" width="22.28" customWidth="true" style="0"/>
+    <col min="12" max="12" width="18.71" customWidth="true" style="0"/>
+    <col min="13" max="13" width="20.995" customWidth="true" style="0"/>
+    <col min="14" max="14" width="11.711" customWidth="true" style="0"/>
+    <col min="15" max="15" width="17.567" customWidth="true" style="0"/>
+    <col min="16" max="16" width="28.136" customWidth="true" style="0"/>
+    <col min="17" max="17" width="8.141" customWidth="true" style="0"/>
+    <col min="18" max="18" width="26.993" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -614,10 +617,10 @@
         <v>27</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -630,7 +633,7 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H3" s="2">
         <v>100</v>

</xml_diff>